<commit_message>
feat: for createReport module
</commit_message>
<xml_diff>
--- a/report_post_creation_visibility.xlsx
+++ b/report_post_creation_visibility.xlsx
@@ -129,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -177,9 +177,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -563,7 +560,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Test Run Summary — post_creation_visibility  |  2026-06-23 15:26</t>
+          <t>Test Run Summary — post_creation_visibility  |  2026-06-25 09:34</t>
         </is>
       </c>
     </row>
@@ -601,10 +598,10 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="7" t="n">
         <v>0</v>
@@ -668,10 +665,10 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D9" s="12" t="n">
         <v>0</v>
@@ -694,7 +691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -800,10 +797,13 @@
       </c>
       <c r="G2" s="14" t="inlineStr">
         <is>
-          <t>ticket_subject: Server Down
-priority_id: High
-status_id: Open
-dept_id: Technical Support</t>
+          <t>customer: Acme Corp
+user: Alice Smith
+service_type: Breakdown Repair
+department: Technical Support
+priority: High
+subject: Server not responding
+staff_assigned: John Doe</t>
         </is>
       </c>
       <c r="H2" s="14" t="inlineStr"/>
@@ -815,7 +815,7 @@
       <c r="J2" s="14" t="inlineStr"/>
       <c r="K2" s="14" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>D1</t>
         </is>
       </c>
     </row>
@@ -847,16 +847,18 @@
       </c>
       <c r="F3" s="16" t="inlineStr">
         <is>
-          <t>Verify that an agent who is the accountable staff can see the ticket record.</t>
+          <t>Session B user CAN see the record when staff_assigned is the agent.</t>
         </is>
       </c>
       <c r="G3" s="16" t="inlineStr">
         <is>
-          <t>ticket_subject: Server Down
-priority_id: High
-status_id: Open
-dept_id: Technical Support
-accountable_staff_id: John Doe</t>
+          <t>customer: Acme Corp
+user: Alice Smith
+service_type: Breakdown Repair
+department: Technical Support
+staff_assigned: John Doe
+priority: High
+subject: Test Subject</t>
         </is>
       </c>
       <c r="H3" s="16" t="inlineStr"/>
@@ -900,15 +902,18 @@
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
-          <t>Verify that an agent who is in the same department as the ticket can see the ticket record.</t>
+          <t>Session B user CAN see the record when staff_accountable is the agent.</t>
         </is>
       </c>
       <c r="G4" s="14" t="inlineStr">
         <is>
-          <t>ticket_subject: Network Issue
-priority_id: Normal
-status_id: In Progress
-dept_id: Technical Support</t>
+          <t>customer: Acme Corp
+user: Alice Smith
+service_type: Breakdown Repair
+department: Technical Support
+staff_accountable: John Doe
+priority: High
+subject: Test Subject</t>
         </is>
       </c>
       <c r="H4" s="14" t="inlineStr"/>
@@ -952,28 +957,83 @@
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>Verify that an agent who is not the accountable staff and not in the same department cannot see the ticket record.</t>
+          <t>Session B user CAN see the record when department has ticket.view permission and agent is manager/admin.</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>ticket_subject: Power Outage
-priority_id: Low
-status_id: Closed
-dept_id: Electrical
-accountable_staff_id: Jane Smith</t>
+          <t>customer: Acme Corp
+user: Alice Smith
+service_type: Breakdown Repair
+department: Electrical
+priority: High
+subject: Test Subject</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr"/>
-      <c r="I5" s="17" t="inlineStr">
-        <is>
-          <t>fail</t>
+      <c r="I5" s="15" t="inlineStr">
+        <is>
+          <t>pass</t>
         </is>
       </c>
       <c r="J5" s="16" t="inlineStr"/>
       <c r="K5" s="16" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>TC005</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>post_creation_visibility</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>post_creation_visibility</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>multi_session</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Session B user CANNOT see the record when conditions are not met.</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>customer: Acme Corp
+user: Alice Smith
+service_type: Breakdown Repair
+department: Technical Support
+priority: High
+subject: Test Subject</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr"/>
+      <c r="I6" s="15" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr"/>
+      <c r="K6" s="14" t="inlineStr">
+        <is>
+          <t>D1, D2, D3</t>
         </is>
       </c>
     </row>
@@ -989,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1091,10 +1151,13 @@
       </c>
       <c r="E2" s="14" t="inlineStr">
         <is>
-          <t>ticket_subject: Server Down
-priority_id: High
-status_id: Open
-dept_id: Technical Support</t>
+          <t>customer: Acme Corp
+user: Alice Smith
+service_type: Breakdown Repair
+department: Technical Support
+priority: High
+subject: Server not responding
+staff_assigned: John Doe</t>
         </is>
       </c>
       <c r="F2" s="14" t="inlineStr">
@@ -1102,7 +1165,7 @@
           <t>pass</t>
         </is>
       </c>
-      <c r="G2" s="18" t="inlineStr">
+      <c r="G2" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1110,10 +1173,10 @@
       <c r="H2" s="14" t="inlineStr"/>
       <c r="I2" s="14" t="inlineStr">
         <is>
-          <t>Ticket 122 visible to Session B (agent)</t>
-        </is>
-      </c>
-      <c r="J2" s="18" t="inlineStr">
+          <t>Ticket 234 visible to Session B (John Doe)</t>
+        </is>
+      </c>
+      <c r="J2" s="17" t="inlineStr">
         <is>
           <t>✓ PASS</t>
         </is>
@@ -1121,7 +1184,7 @@
       <c r="K2" s="14" t="inlineStr"/>
       <c r="L2" s="14" t="inlineStr">
         <is>
-          <t>2026-06-23 15:26</t>
+          <t>2026-06-25 09:34</t>
         </is>
       </c>
     </row>
@@ -1143,16 +1206,18 @@
       </c>
       <c r="D3" s="16" t="inlineStr">
         <is>
-          <t>Verify that an agent who is the accountable staff can see the ticket record.</t>
+          <t>Session B user CAN see the record when staff_assigned is the agent.</t>
         </is>
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
-          <t>ticket_subject: Server Down
-priority_id: High
-status_id: Open
-dept_id: Technical Support
-accountable_staff_id: John Doe</t>
+          <t>customer: Acme Corp
+user: Alice Smith
+service_type: Breakdown Repair
+department: Technical Support
+staff_assigned: John Doe
+priority: High
+subject: Test Subject</t>
         </is>
       </c>
       <c r="F3" s="16" t="inlineStr">
@@ -1160,7 +1225,7 @@
           <t>pass</t>
         </is>
       </c>
-      <c r="G3" s="18" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1168,10 +1233,10 @@
       <c r="H3" s="16" t="inlineStr"/>
       <c r="I3" s="16" t="inlineStr">
         <is>
-          <t>Ticket 123 visible to Session B (John Doe)</t>
-        </is>
-      </c>
-      <c r="J3" s="18" t="inlineStr">
+          <t>Ticket 235 visible to Session B (John Doe)</t>
+        </is>
+      </c>
+      <c r="J3" s="17" t="inlineStr">
         <is>
           <t>✓ PASS</t>
         </is>
@@ -1179,7 +1244,7 @@
       <c r="K3" s="16" t="inlineStr"/>
       <c r="L3" s="16" t="inlineStr">
         <is>
-          <t>2026-06-23 15:26</t>
+          <t>2026-06-25 09:34</t>
         </is>
       </c>
     </row>
@@ -1201,15 +1266,18 @@
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>Verify that an agent who is in the same department as the ticket can see the ticket record.</t>
+          <t>Session B user CAN see the record when staff_accountable is the agent.</t>
         </is>
       </c>
       <c r="E4" s="14" t="inlineStr">
         <is>
-          <t>ticket_subject: Network Issue
-priority_id: Normal
-status_id: In Progress
-dept_id: Technical Support</t>
+          <t>customer: Acme Corp
+user: Alice Smith
+service_type: Breakdown Repair
+department: Technical Support
+staff_accountable: John Doe
+priority: High
+subject: Test Subject</t>
         </is>
       </c>
       <c r="F4" s="14" t="inlineStr">
@@ -1217,7 +1285,7 @@
           <t>pass</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1225,10 +1293,10 @@
       <c r="H4" s="14" t="inlineStr"/>
       <c r="I4" s="14" t="inlineStr">
         <is>
-          <t>Ticket 124 visible to Session B (Liam Hughes)</t>
-        </is>
-      </c>
-      <c r="J4" s="18" t="inlineStr">
+          <t>Ticket 237 visible to Session B (John Doe)</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="inlineStr">
         <is>
           <t>✓ PASS</t>
         </is>
@@ -1236,7 +1304,7 @@
       <c r="K4" s="14" t="inlineStr"/>
       <c r="L4" s="14" t="inlineStr">
         <is>
-          <t>2026-06-23 15:26</t>
+          <t>2026-06-25 09:34</t>
         </is>
       </c>
     </row>
@@ -1258,24 +1326,25 @@
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>Verify that an agent who is not the accountable staff and not in the same department cannot see the ticket record.</t>
+          <t>Session B user CAN see the record when department has ticket.view permission and agent is manager/admin.</t>
         </is>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>ticket_subject: Power Outage
-priority_id: Low
-status_id: Closed
-dept_id: Electrical
-accountable_staff_id: Jane Smith</t>
+          <t>customer: Acme Corp
+user: Alice Smith
+service_type: Breakdown Repair
+department: Electrical
+priority: High
+subject: Test Subject</t>
         </is>
       </c>
       <c r="F5" s="16" t="inlineStr">
         <is>
-          <t>fail</t>
-        </is>
-      </c>
-      <c r="G5" s="18" t="inlineStr">
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
@@ -1283,10 +1352,10 @@
       <c r="H5" s="16" t="inlineStr"/>
       <c r="I5" s="16" t="inlineStr">
         <is>
-          <t>Ticket 125 visible to Session B (Carlos Silva)</t>
-        </is>
-      </c>
-      <c r="J5" s="18" t="inlineStr">
+          <t>Ticket 238 visible to Session B (John Doe)</t>
+        </is>
+      </c>
+      <c r="J5" s="17" t="inlineStr">
         <is>
           <t>✓ PASS</t>
         </is>
@@ -1294,7 +1363,66 @@
       <c r="K5" s="16" t="inlineStr"/>
       <c r="L5" s="16" t="inlineStr">
         <is>
-          <t>2026-06-23 15:26</t>
+          <t>2026-06-25 09:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>TC005</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>post_creation_visibility</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>agent</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Session B user CANNOT see the record when conditions are not met.</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>customer: Acme Corp
+user: Alice Smith
+service_type: Breakdown Repair
+department: Technical Support
+priority: High
+subject: Test Subject</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="G6" s="17" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr"/>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>Ticket 239 correctly hidden to Session B (Liam Hughes)</t>
+        </is>
+      </c>
+      <c r="J6" s="17" t="inlineStr">
+        <is>
+          <t>✓ PASS</t>
+        </is>
+      </c>
+      <c r="K6" s="14" t="inlineStr"/>
+      <c r="L6" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-25 09:34</t>
         </is>
       </c>
     </row>

</xml_diff>